<commit_message>
mod: property break attribute set to INVALID
</commit_message>
<xml_diff>
--- a/ContinuationProject/WorkingFolder/BLUEPRINTS-13_DATA_PROPS.xlsx
+++ b/ContinuationProject/WorkingFolder/BLUEPRINTS-13_DATA_PROPS.xlsx
@@ -5,13 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\DISCDEXPI\ContinuationProject\WorkingFolder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mso\Desktop\todo\discII\github\DISCDEXPI\ContinuationProject\WorkingFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C7F0B1-FC00-4CAA-B787-8A4012BC0803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F260D5-1D46-41AA-A8F0-D3CA1889F052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{D454660A-399F-40A5-B0DC-958E447D7F13}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D454660A-399F-40A5-B0DC-958E447D7F13}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA_PROPS" sheetId="2" r:id="rId1"/>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="129">
   <si>
     <t>Core.Diagram.AttributeRepresentation.AttributeName</t>
   </si>
@@ -418,6 +417,9 @@
   </si>
   <si>
     <t>VALID</t>
+  </si>
+  <si>
+    <t>INVALID</t>
   </si>
 </sst>
 </file>
@@ -457,7 +459,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -758,13 +760,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B126"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="97.42578125" customWidth="1"/>
+    <col min="1" max="1" width="97.44140625" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -772,7 +774,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -780,7 +782,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -788,7 +790,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -796,7 +798,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -804,7 +806,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -812,7 +814,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -820,7 +822,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -828,7 +830,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -836,7 +838,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -844,7 +846,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -852,7 +854,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -860,7 +862,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -868,7 +870,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -876,7 +878,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -884,7 +886,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -892,7 +894,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -900,7 +902,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -908,7 +910,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -916,7 +918,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -924,7 +926,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -932,7 +934,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -940,7 +942,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -948,7 +950,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -956,7 +958,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -964,7 +966,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -972,7 +974,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -980,7 +982,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -988,7 +990,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -996,7 +998,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -1004,7 +1006,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -1012,7 +1014,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -1020,7 +1022,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -1028,7 +1030,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -1036,7 +1038,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -1044,7 +1046,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -1052,7 +1054,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -1060,7 +1062,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -1068,7 +1070,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -1076,7 +1078,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -1084,7 +1086,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -1092,7 +1094,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -1100,7 +1102,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -1108,7 +1110,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -1116,7 +1118,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -1124,7 +1126,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -1132,7 +1134,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>46</v>
       </c>
@@ -1140,7 +1142,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -1148,7 +1150,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -1156,7 +1158,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>49</v>
       </c>
@@ -1164,7 +1166,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>50</v>
       </c>
@@ -1172,7 +1174,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>51</v>
       </c>
@@ -1180,7 +1182,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>52</v>
       </c>
@@ -1188,7 +1190,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>53</v>
       </c>
@@ -1196,7 +1198,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>54</v>
       </c>
@@ -1204,7 +1206,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>55</v>
       </c>
@@ -1212,7 +1214,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>56</v>
       </c>
@@ -1220,7 +1222,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>57</v>
       </c>
@@ -1228,7 +1230,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>58</v>
       </c>
@@ -1236,7 +1238,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -1244,7 +1246,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>60</v>
       </c>
@@ -1252,7 +1254,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>61</v>
       </c>
@@ -1260,7 +1262,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>62</v>
       </c>
@@ -1268,7 +1270,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>63</v>
       </c>
@@ -1276,7 +1278,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>64</v>
       </c>
@@ -1284,7 +1286,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>65</v>
       </c>
@@ -1292,7 +1294,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>66</v>
       </c>
@@ -1300,7 +1302,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>67</v>
       </c>
@@ -1308,7 +1310,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>68</v>
       </c>
@@ -1316,7 +1318,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>69</v>
       </c>
@@ -1324,7 +1326,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -1332,7 +1334,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -1340,7 +1342,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>72</v>
       </c>
@@ -1348,7 +1350,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -1356,7 +1358,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>74</v>
       </c>
@@ -1364,7 +1366,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>75</v>
       </c>
@@ -1372,7 +1374,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>76</v>
       </c>
@@ -1380,7 +1382,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>77</v>
       </c>
@@ -1388,7 +1390,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>78</v>
       </c>
@@ -1396,7 +1398,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>79</v>
       </c>
@@ -1404,7 +1406,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>80</v>
       </c>
@@ -1412,7 +1414,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>81</v>
       </c>
@@ -1420,7 +1422,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>82</v>
       </c>
@@ -1428,7 +1430,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -1436,7 +1438,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>84</v>
       </c>
@@ -1444,7 +1446,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>85</v>
       </c>
@@ -1452,7 +1454,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>86</v>
       </c>
@@ -1460,7 +1462,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>87</v>
       </c>
@@ -1468,7 +1470,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>88</v>
       </c>
@@ -1476,7 +1478,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>89</v>
       </c>
@@ -1484,7 +1486,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>90</v>
       </c>
@@ -1492,7 +1494,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>91</v>
       </c>
@@ -1500,7 +1502,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>92</v>
       </c>
@@ -1508,7 +1510,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>93</v>
       </c>
@@ -1516,7 +1518,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>94</v>
       </c>
@@ -1524,7 +1526,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>95</v>
       </c>
@@ -1532,7 +1534,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>96</v>
       </c>
@@ -1540,7 +1542,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>97</v>
       </c>
@@ -1548,7 +1550,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>98</v>
       </c>
@@ -1556,7 +1558,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>99</v>
       </c>
@@ -1564,7 +1566,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>100</v>
       </c>
@@ -1572,7 +1574,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>101</v>
       </c>
@@ -1580,7 +1582,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>102</v>
       </c>
@@ -1588,7 +1590,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>103</v>
       </c>
@@ -1596,7 +1598,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>104</v>
       </c>
@@ -1604,7 +1606,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>105</v>
       </c>
@@ -1612,7 +1614,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>106</v>
       </c>
@@ -1620,7 +1622,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>107</v>
       </c>
@@ -1628,7 +1630,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>108</v>
       </c>
@@ -1636,7 +1638,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>109</v>
       </c>
@@ -1644,7 +1646,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>110</v>
       </c>
@@ -1652,7 +1654,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>111</v>
       </c>
@@ -1660,7 +1662,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>112</v>
       </c>
@@ -1668,7 +1670,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>113</v>
       </c>
@@ -1676,7 +1678,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>114</v>
       </c>
@@ -1684,15 +1686,15 @@
         <v>127</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>116</v>
       </c>
@@ -1700,7 +1702,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>117</v>
       </c>
@@ -1708,7 +1710,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>118</v>
       </c>
@@ -1716,7 +1718,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>119</v>
       </c>
@@ -1724,7 +1726,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>120</v>
       </c>
@@ -1732,7 +1734,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>121</v>
       </c>
@@ -1740,7 +1742,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>122</v>
       </c>
@@ -1748,7 +1750,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>123</v>
       </c>
@@ -1756,7 +1758,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>124</v>
       </c>
@@ -1764,7 +1766,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>125</v>
       </c>

</xml_diff>

<commit_message>
mod: unique usage of string "NOT VALID"
</commit_message>
<xml_diff>
--- a/ContinuationProject/WorkingFolder/BLUEPRINTS-13_DATA_PROPS.xlsx
+++ b/ContinuationProject/WorkingFolder/BLUEPRINTS-13_DATA_PROPS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mso\Desktop\todo\discII\github\DISCDEXPI\ContinuationProject\WorkingFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F260D5-1D46-41AA-A8F0-D3CA1889F052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C696E6A7-F767-4F15-AC0A-E832897B0E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D454660A-399F-40A5-B0DC-958E447D7F13}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="128">
   <si>
     <t>Core.Diagram.AttributeRepresentation.AttributeName</t>
   </si>
@@ -417,9 +417,6 @@
   </si>
   <si>
     <t>VALID</t>
-  </si>
-  <si>
-    <t>INVALID</t>
   </si>
 </sst>
 </file>
@@ -1691,7 +1688,7 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>